<commit_message>
network effect exposed for SA
</commit_message>
<xml_diff>
--- a/All_perf.xlsx
+++ b/All_perf.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10917"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10329"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ttdkoc/Documents/dev/workspaces/python/copt/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{918BE3DF-5DF5-4943-91DA-9F177CA705BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7ED7288C-5F95-D54B-9213-6266013E6BE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20440" activeTab="8" xr2:uid="{544C10BC-9448-4CAA-97CB-C174D9523FCA}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20440" activeTab="6" xr2:uid="{544C10BC-9448-4CAA-97CB-C174D9523FCA}"/>
   </bookViews>
   <sheets>
     <sheet name="loose channel" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="52">
   <si>
     <t>Exact</t>
   </si>
@@ -198,6 +198,15 @@
   <si>
     <t>SA+Agg+
 Grdy©</t>
+  </si>
+  <si>
+    <t>Exact/NO - NET</t>
+  </si>
+  <si>
+    <t>Net Ratio</t>
+  </si>
+  <si>
+    <t>SA+Greed With Alg-C/NO - NET</t>
   </si>
 </sst>
 </file>
@@ -497,6 +506,14 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -527,14 +544,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Bad" xfId="2" builtinId="27"/>
@@ -1384,7 +1393,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-TR"/>
+          <a:endParaRPr lang="tr-TR"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -16910,27 +16919,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:18" x14ac:dyDescent="0.2">
-      <c r="B1" s="46" t="s">
+      <c r="B1" s="50" t="s">
         <v>6</v>
       </c>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="F1" s="46" t="s">
+      <c r="C1" s="50"/>
+      <c r="D1" s="50"/>
+      <c r="F1" s="50" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="46"/>
-      <c r="H1" s="46"/>
-      <c r="J1" s="46" t="s">
+      <c r="G1" s="50"/>
+      <c r="H1" s="50"/>
+      <c r="J1" s="50" t="s">
         <v>5</v>
       </c>
-      <c r="K1" s="46"/>
-      <c r="L1" s="46"/>
-      <c r="N1" s="46" t="s">
+      <c r="K1" s="50"/>
+      <c r="L1" s="50"/>
+      <c r="N1" s="50" t="s">
         <v>0</v>
       </c>
-      <c r="O1" s="46"/>
-      <c r="Q1" s="46"/>
-      <c r="R1" s="46"/>
+      <c r="O1" s="50"/>
+      <c r="Q1" s="50"/>
+      <c r="R1" s="50"/>
     </row>
     <row r="2" spans="2:18" x14ac:dyDescent="0.2">
       <c r="B2">
@@ -18881,41 +18890,41 @@
       <c r="V1" s="33"/>
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A2" s="48" t="s">
+      <c r="A2" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="52" t="s">
+      <c r="B2" s="56" t="s">
         <v>27</v>
       </c>
-      <c r="C2" s="52"/>
-      <c r="D2" s="52"/>
+      <c r="C2" s="56"/>
+      <c r="D2" s="56"/>
       <c r="E2" s="32"/>
-      <c r="F2" s="50" t="s">
+      <c r="F2" s="54" t="s">
         <v>28</v>
       </c>
-      <c r="G2" s="50"/>
-      <c r="H2" s="50"/>
-      <c r="I2" s="50"/>
-      <c r="L2" s="48" t="s">
+      <c r="G2" s="54"/>
+      <c r="H2" s="54"/>
+      <c r="I2" s="54"/>
+      <c r="L2" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="M2" s="51" t="s">
+      <c r="M2" s="55" t="s">
         <v>27</v>
       </c>
-      <c r="N2" s="51"/>
-      <c r="O2" s="51"/>
-      <c r="P2" s="51"/>
+      <c r="N2" s="55"/>
+      <c r="O2" s="55"/>
+      <c r="P2" s="55"/>
       <c r="Q2" s="32"/>
-      <c r="R2" s="50" t="s">
+      <c r="R2" s="54" t="s">
         <v>28</v>
       </c>
-      <c r="S2" s="50"/>
-      <c r="T2" s="50"/>
-      <c r="U2" s="50"/>
-      <c r="V2" s="50"/>
+      <c r="S2" s="54"/>
+      <c r="T2" s="54"/>
+      <c r="U2" s="54"/>
+      <c r="V2" s="54"/>
     </row>
     <row r="3" spans="1:22" ht="32" x14ac:dyDescent="0.2">
-      <c r="A3" s="49"/>
+      <c r="A3" s="53"/>
       <c r="B3" s="26" t="s">
         <v>31</v>
       </c>
@@ -18938,7 +18947,7 @@
       <c r="I3" s="26" t="s">
         <v>33</v>
       </c>
-      <c r="L3" s="49"/>
+      <c r="L3" s="53"/>
       <c r="M3" s="27" t="s">
         <v>37</v>
       </c>
@@ -20163,24 +20172,24 @@
       <c r="I25" s="33"/>
     </row>
     <row r="26" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="A26" s="48" t="s">
+      <c r="A26" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="B26" s="52" t="s">
+      <c r="B26" s="56" t="s">
         <v>27</v>
       </c>
-      <c r="C26" s="52"/>
-      <c r="D26" s="52"/>
+      <c r="C26" s="56"/>
+      <c r="D26" s="56"/>
       <c r="E26" s="32"/>
-      <c r="F26" s="50" t="s">
+      <c r="F26" s="54" t="s">
         <v>28</v>
       </c>
-      <c r="G26" s="50"/>
-      <c r="H26" s="50"/>
-      <c r="I26" s="50"/>
+      <c r="G26" s="54"/>
+      <c r="H26" s="54"/>
+      <c r="I26" s="54"/>
     </row>
     <row r="27" spans="1:22" ht="32" x14ac:dyDescent="0.2">
-      <c r="A27" s="49"/>
+      <c r="A27" s="53"/>
       <c r="B27" s="26" t="s">
         <v>31</v>
       </c>
@@ -20798,37 +20807,37 @@
       <c r="S1" s="34"/>
     </row>
     <row r="2" spans="1:19" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="53" t="s">
+      <c r="A2" s="57" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="51" t="s">
+      <c r="B2" s="55" t="s">
         <v>34</v>
       </c>
-      <c r="C2" s="51"/>
+      <c r="C2" s="55"/>
       <c r="D2" s="32"/>
-      <c r="E2" s="51" t="s">
+      <c r="E2" s="55" t="s">
         <v>28</v>
       </c>
-      <c r="F2" s="51"/>
-      <c r="G2" s="51"/>
-      <c r="K2" s="53" t="s">
+      <c r="F2" s="55"/>
+      <c r="G2" s="55"/>
+      <c r="K2" s="57" t="s">
         <v>1</v>
       </c>
-      <c r="L2" s="55" t="s">
+      <c r="L2" s="59" t="s">
         <v>42</v>
       </c>
-      <c r="M2" s="51"/>
-      <c r="N2" s="51"/>
+      <c r="M2" s="55"/>
+      <c r="N2" s="55"/>
       <c r="O2" s="32"/>
-      <c r="P2" s="51" t="s">
+      <c r="P2" s="55" t="s">
         <v>28</v>
       </c>
-      <c r="Q2" s="51"/>
-      <c r="R2" s="51"/>
-      <c r="S2" s="51"/>
+      <c r="Q2" s="55"/>
+      <c r="R2" s="55"/>
+      <c r="S2" s="55"/>
     </row>
     <row r="3" spans="1:19" ht="35" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="54"/>
+      <c r="A3" s="58"/>
       <c r="B3" s="27" t="s">
         <v>31</v>
       </c>
@@ -20845,7 +20854,7 @@
       <c r="G3" s="27" t="s">
         <v>33</v>
       </c>
-      <c r="K3" s="54"/>
+      <c r="K3" s="58"/>
       <c r="L3" s="27" t="s">
         <v>37</v>
       </c>
@@ -23678,29 +23687,29 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A1" s="46" t="s">
+      <c r="A1" s="50" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="E1" s="46" t="s">
+      <c r="B1" s="50"/>
+      <c r="C1" s="50"/>
+      <c r="E1" s="50" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="46"/>
-      <c r="G1" s="46"/>
-      <c r="I1" s="46" t="s">
+      <c r="F1" s="50"/>
+      <c r="G1" s="50"/>
+      <c r="I1" s="50" t="s">
         <v>5</v>
       </c>
-      <c r="J1" s="46"/>
-      <c r="K1" s="46"/>
-      <c r="M1" s="46" t="s">
+      <c r="J1" s="50"/>
+      <c r="K1" s="50"/>
+      <c r="M1" s="50" t="s">
         <v>0</v>
       </c>
-      <c r="N1" s="46"/>
-      <c r="P1" s="46" t="s">
+      <c r="N1" s="50"/>
+      <c r="P1" s="50" t="s">
         <v>8</v>
       </c>
-      <c r="Q1" s="46"/>
+      <c r="Q1" s="50"/>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A2">
@@ -26168,30 +26177,30 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:22" x14ac:dyDescent="0.2">
-      <c r="D2" s="46" t="s">
+      <c r="D2" s="50" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="46"/>
-      <c r="F2" s="46"/>
-      <c r="G2" s="46"/>
-      <c r="I2" s="46" t="s">
+      <c r="E2" s="50"/>
+      <c r="F2" s="50"/>
+      <c r="G2" s="50"/>
+      <c r="I2" s="50" t="s">
         <v>16</v>
       </c>
-      <c r="J2" s="46"/>
-      <c r="K2" s="46"/>
-      <c r="L2" s="46"/>
-      <c r="N2" s="46" t="s">
+      <c r="J2" s="50"/>
+      <c r="K2" s="50"/>
+      <c r="L2" s="50"/>
+      <c r="N2" s="50" t="s">
         <v>17</v>
       </c>
-      <c r="O2" s="46"/>
-      <c r="P2" s="46"/>
-      <c r="Q2" s="46"/>
-      <c r="S2" s="46" t="s">
+      <c r="O2" s="50"/>
+      <c r="P2" s="50"/>
+      <c r="Q2" s="50"/>
+      <c r="S2" s="50" t="s">
         <v>18</v>
       </c>
-      <c r="T2" s="46"/>
-      <c r="U2" s="46"/>
-      <c r="V2" s="46"/>
+      <c r="T2" s="50"/>
+      <c r="U2" s="50"/>
+      <c r="V2" s="50"/>
     </row>
     <row r="3" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
@@ -27066,7 +27075,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06C03F23-5B48-E740-AE12-B3F8383D5054}">
-  <dimension ref="A2:AM26"/>
+  <dimension ref="A2:AS27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="8.6640625" bestFit="1" customWidth="1"/>
@@ -27105,51 +27114,65 @@
     <col min="37" max="37" width="7.1640625" bestFit="1" customWidth="1"/>
     <col min="38" max="38" width="6.1640625" customWidth="1"/>
     <col min="39" max="39" width="4" style="19" customWidth="1"/>
+    <col min="40" max="40" width="18" customWidth="1"/>
+    <col min="41" max="41" width="8.1640625" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="4" style="19" customWidth="1"/>
+    <col min="43" max="43" width="12.83203125" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="8.1640625" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="11.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:38" x14ac:dyDescent="0.2">
-      <c r="E2" s="46" t="s">
+    <row r="2" spans="1:45" x14ac:dyDescent="0.2">
+      <c r="E2" s="50" t="s">
         <v>0</v>
       </c>
-      <c r="F2" s="46"/>
-      <c r="G2" s="46"/>
-      <c r="H2" s="46"/>
+      <c r="F2" s="50"/>
+      <c r="G2" s="50"/>
+      <c r="H2" s="50"/>
       <c r="I2" s="18"/>
-      <c r="K2" s="46" t="s">
+      <c r="K2" s="50" t="s">
         <v>16</v>
       </c>
-      <c r="L2" s="46"/>
-      <c r="M2" s="46"/>
-      <c r="N2" s="46"/>
-      <c r="O2" s="46"/>
+      <c r="L2" s="50"/>
+      <c r="M2" s="50"/>
+      <c r="N2" s="50"/>
+      <c r="O2" s="50"/>
       <c r="P2" s="18"/>
       <c r="Q2" s="18"/>
-      <c r="S2" s="46" t="s">
+      <c r="S2" s="50" t="s">
         <v>17</v>
       </c>
-      <c r="T2" s="46"/>
-      <c r="U2" s="46"/>
-      <c r="V2" s="46"/>
-      <c r="W2" s="46"/>
+      <c r="T2" s="50"/>
+      <c r="U2" s="50"/>
+      <c r="V2" s="50"/>
+      <c r="W2" s="50"/>
       <c r="X2" s="18"/>
       <c r="Y2" s="18"/>
-      <c r="AA2" s="46" t="s">
+      <c r="AA2" s="50" t="s">
         <v>18</v>
       </c>
-      <c r="AB2" s="46"/>
-      <c r="AC2" s="46"/>
-      <c r="AD2" s="46"/>
-      <c r="AE2" s="46"/>
+      <c r="AB2" s="50"/>
+      <c r="AC2" s="50"/>
+      <c r="AD2" s="50"/>
+      <c r="AE2" s="50"/>
       <c r="AF2" s="18"/>
-      <c r="AH2" s="46" t="s">
+      <c r="AH2" s="50" t="s">
         <v>36</v>
       </c>
-      <c r="AI2" s="46"/>
-      <c r="AJ2" s="46"/>
-      <c r="AK2" s="46"/>
-      <c r="AL2" s="46"/>
-    </row>
-    <row r="3" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AI2" s="50"/>
+      <c r="AJ2" s="50"/>
+      <c r="AK2" s="50"/>
+      <c r="AL2" s="50"/>
+      <c r="AN2" s="50" t="s">
+        <v>49</v>
+      </c>
+      <c r="AO2" s="50"/>
+      <c r="AQ2" s="50" t="s">
+        <v>51</v>
+      </c>
+      <c r="AR2" s="50"/>
+    </row>
+    <row r="3" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -27249,8 +27272,20 @@
       <c r="AL3" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="4" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AN3" t="s">
+        <v>11</v>
+      </c>
+      <c r="AO3" t="s">
+        <v>50</v>
+      </c>
+      <c r="AQ3" t="s">
+        <v>11</v>
+      </c>
+      <c r="AR3" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="4" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>0</v>
       </c>
@@ -27365,7 +27400,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="5" spans="1:38" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>1</v>
       </c>
@@ -27385,7 +27420,7 @@
         <v>97</v>
       </c>
       <c r="H5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I5">
         <f t="shared" ref="I5:I19" si="8">F5/G5</f>
@@ -27479,8 +27514,22 @@
         <f t="shared" ref="AL5:AL26" si="13">AI5/AJ5</f>
         <v>55.684210526315788</v>
       </c>
-    </row>
-    <row r="6" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AN5">
+        <v>4263</v>
+      </c>
+      <c r="AO5" s="4">
+        <f>F5/AN5</f>
+        <v>1.264367816091954</v>
+      </c>
+      <c r="AQ5">
+        <v>4851</v>
+      </c>
+      <c r="AR5" s="4">
+        <f>AI5/AQ5</f>
+        <v>1.090496804782519</v>
+      </c>
+    </row>
+    <row r="6" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>2</v>
       </c>
@@ -27500,7 +27549,7 @@
         <v>255</v>
       </c>
       <c r="H6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I6">
         <f t="shared" si="8"/>
@@ -27594,8 +27643,22 @@
         <f t="shared" si="13"/>
         <v>28.677685950413224</v>
       </c>
-    </row>
-    <row r="7" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AN6">
+        <v>3290</v>
+      </c>
+      <c r="AO6" s="4">
+        <f>F6/AN6</f>
+        <v>2.2158054711246202</v>
+      </c>
+      <c r="AQ6">
+        <v>3170</v>
+      </c>
+      <c r="AR6" s="4">
+        <f t="shared" ref="AR6:AR26" si="14">AI6/AQ6</f>
+        <v>2.189274447949527</v>
+      </c>
+    </row>
+    <row r="7" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>3</v>
       </c>
@@ -27615,7 +27678,7 @@
         <v>499</v>
       </c>
       <c r="H7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I7">
         <f t="shared" si="8"/>
@@ -27709,8 +27772,22 @@
         <f t="shared" si="13"/>
         <v>49.087866108786613</v>
       </c>
-    </row>
-    <row r="8" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AN7">
+        <v>12316</v>
+      </c>
+      <c r="AO7" s="4">
+        <f>F7/AN7</f>
+        <v>1.9870087690808704</v>
+      </c>
+      <c r="AQ7">
+        <v>7659</v>
+      </c>
+      <c r="AR7" s="4">
+        <f t="shared" si="14"/>
+        <v>3.0635853244548898</v>
+      </c>
+    </row>
+    <row r="8" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>4</v>
       </c>
@@ -27824,8 +27901,22 @@
         <f t="shared" si="13"/>
         <v>24.095697980684811</v>
       </c>
-    </row>
-    <row r="9" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AN8">
+        <v>17578</v>
+      </c>
+      <c r="AO8" s="4">
+        <f>F8/AN8</f>
+        <v>1.6695869837296622</v>
+      </c>
+      <c r="AQ8">
+        <v>8318</v>
+      </c>
+      <c r="AR8" s="4">
+        <f t="shared" si="14"/>
+        <v>3.2994710266891079</v>
+      </c>
+    </row>
+    <row r="9" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>5</v>
       </c>
@@ -27939,8 +28030,22 @@
         <f t="shared" si="13"/>
         <v>57.940880503144655</v>
       </c>
-    </row>
-    <row r="10" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AN9">
+        <v>43100</v>
+      </c>
+      <c r="AO9" s="4">
+        <f>F9/AN9</f>
+        <v>2.3034802784222737</v>
+      </c>
+      <c r="AQ9">
+        <v>32504</v>
+      </c>
+      <c r="AR9" s="4">
+        <f t="shared" si="14"/>
+        <v>2.8342973172532613</v>
+      </c>
+    </row>
+    <row r="10" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>6</v>
       </c>
@@ -28054,8 +28159,22 @@
         <f t="shared" si="13"/>
         <v>13.792730419731718</v>
       </c>
-    </row>
-    <row r="11" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AN10">
+        <v>23591</v>
+      </c>
+      <c r="AO10" s="4">
+        <f>F10/AN10</f>
+        <v>1.4001526005680132</v>
+      </c>
+      <c r="AQ10">
+        <v>17749</v>
+      </c>
+      <c r="AR10" s="4">
+        <f t="shared" si="14"/>
+        <v>1.7958758239900841</v>
+      </c>
+    </row>
+    <row r="11" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>7</v>
       </c>
@@ -28169,8 +28288,22 @@
         <f t="shared" si="13"/>
         <v>23.729269385925594</v>
       </c>
-    </row>
-    <row r="12" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AN11">
+        <v>60450</v>
+      </c>
+      <c r="AO11" s="4">
+        <f>F11/AN11</f>
+        <v>1.9103887510339124</v>
+      </c>
+      <c r="AQ11">
+        <v>22396</v>
+      </c>
+      <c r="AR11" s="4">
+        <f t="shared" si="14"/>
+        <v>4.7276299339167709</v>
+      </c>
+    </row>
+    <row r="12" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>8</v>
       </c>
@@ -28284,8 +28417,22 @@
         <f t="shared" si="13"/>
         <v>39.393946188340806</v>
       </c>
-    </row>
-    <row r="13" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AN12">
+        <v>168828</v>
+      </c>
+      <c r="AO12" s="4">
+        <f>F12/AN12</f>
+        <v>2.194612268107186</v>
+      </c>
+      <c r="AQ12">
+        <v>109494</v>
+      </c>
+      <c r="AR12" s="4">
+        <f t="shared" si="14"/>
+        <v>3.20925347507626</v>
+      </c>
+    </row>
+    <row r="13" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>9</v>
       </c>
@@ -28399,8 +28546,22 @@
         <f t="shared" si="13"/>
         <v>59.157081063761616</v>
       </c>
-    </row>
-    <row r="14" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AN13">
+        <v>478828</v>
+      </c>
+      <c r="AO13" s="4">
+        <f>F13/AN13</f>
+        <v>1.6686743465294427</v>
+      </c>
+      <c r="AQ13">
+        <v>226956</v>
+      </c>
+      <c r="AR13" s="4">
+        <f t="shared" si="14"/>
+        <v>3.2540095877615043</v>
+      </c>
+    </row>
+    <row r="14" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>10</v>
       </c>
@@ -28514,8 +28675,23 @@
         <f t="shared" si="13"/>
         <v>52.598314268512944</v>
       </c>
-    </row>
-    <row r="15" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AN14">
+        <v>420398</v>
+      </c>
+      <c r="AO14" s="4">
+        <f>F14/AN14</f>
+        <v>2.1977245372242495</v>
+      </c>
+      <c r="AQ14">
+        <v>390761</v>
+      </c>
+      <c r="AR14" s="4">
+        <f t="shared" si="14"/>
+        <v>2.2357860687223137</v>
+      </c>
+      <c r="AS14" s="6"/>
+    </row>
+    <row r="15" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>11</v>
       </c>
@@ -28629,8 +28805,23 @@
         <f t="shared" si="13"/>
         <v>50.422024525126233</v>
       </c>
-    </row>
-    <row r="16" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AN15">
+        <v>444705</v>
+      </c>
+      <c r="AO15" s="4">
+        <f>F15/AN15</f>
+        <v>2.4277194994434512</v>
+      </c>
+      <c r="AQ15">
+        <v>549158</v>
+      </c>
+      <c r="AR15" s="4">
+        <f t="shared" si="14"/>
+        <v>1.9093339257554292</v>
+      </c>
+      <c r="AS15" s="6"/>
+    </row>
+    <row r="16" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>12</v>
       </c>
@@ -28744,8 +28935,23 @@
         <f t="shared" si="13"/>
         <v>88.592836946277103</v>
       </c>
-    </row>
-    <row r="17" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AN16">
+        <v>882776</v>
+      </c>
+      <c r="AO16" s="4">
+        <f>F16/AN16</f>
+        <v>4.000458780030268</v>
+      </c>
+      <c r="AQ16">
+        <v>985185</v>
+      </c>
+      <c r="AR16" s="4">
+        <f t="shared" si="14"/>
+        <v>3.4347782396199698</v>
+      </c>
+      <c r="AS16" s="6"/>
+    </row>
+    <row r="17" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>13</v>
       </c>
@@ -28859,8 +29065,23 @@
         <f t="shared" si="13"/>
         <v>102.40332113170136</v>
       </c>
-    </row>
-    <row r="18" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AN17">
+        <v>1143696</v>
+      </c>
+      <c r="AO17" s="4">
+        <f>F17/AN17</f>
+        <v>5.1860774191743264</v>
+      </c>
+      <c r="AQ17">
+        <v>2504407</v>
+      </c>
+      <c r="AR17" s="4">
+        <f t="shared" si="14"/>
+        <v>2.144722882502724</v>
+      </c>
+      <c r="AS17" s="6"/>
+    </row>
+    <row r="18" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>14</v>
       </c>
@@ -28974,8 +29195,23 @@
         <f t="shared" si="13"/>
         <v>115.67040964644707</v>
       </c>
-    </row>
-    <row r="19" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AN18">
+        <v>1690024</v>
+      </c>
+      <c r="AO18" s="4">
+        <f>F18/AN18</f>
+        <v>7.0191855263593892</v>
+      </c>
+      <c r="AQ18">
+        <v>4855080</v>
+      </c>
+      <c r="AR18" s="4">
+        <f t="shared" si="14"/>
+        <v>2.3275218945928802</v>
+      </c>
+      <c r="AS18" s="6"/>
+    </row>
+    <row r="19" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>15</v>
       </c>
@@ -29089,8 +29325,23 @@
         <f t="shared" si="13"/>
         <v>116.87897458572033</v>
       </c>
-    </row>
-    <row r="20" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AN19">
+        <v>4196220</v>
+      </c>
+      <c r="AO19" s="4">
+        <f>F19/AN19</f>
+        <v>3.0721206228462759</v>
+      </c>
+      <c r="AQ19">
+        <v>2798271</v>
+      </c>
+      <c r="AR19" s="4">
+        <f t="shared" si="14"/>
+        <v>4.3454050733470773</v>
+      </c>
+      <c r="AS19" s="6"/>
+    </row>
+    <row r="20" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>16</v>
       </c>
@@ -29175,8 +29426,20 @@
         <f t="shared" si="13"/>
         <v>103.56100666666667</v>
       </c>
-    </row>
-    <row r="21" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AO20" s="4">
+        <f>AVERAGE(AO5:AO19)</f>
+        <v>2.7011575779843926</v>
+      </c>
+      <c r="AQ20">
+        <v>6135807</v>
+      </c>
+      <c r="AR20" s="4">
+        <f>AI20/AQ20</f>
+        <v>2.5317209292925935</v>
+      </c>
+      <c r="AS20" s="6"/>
+    </row>
+    <row r="21" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>17</v>
       </c>
@@ -29261,8 +29524,16 @@
         <f t="shared" si="13"/>
         <v>132.8531759053088</v>
       </c>
-    </row>
-    <row r="22" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AQ21">
+        <v>7276898</v>
+      </c>
+      <c r="AR21" s="4">
+        <f t="shared" si="14"/>
+        <v>3.1157126291999697</v>
+      </c>
+      <c r="AS21" s="6"/>
+    </row>
+    <row r="22" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>18</v>
       </c>
@@ -29347,8 +29618,16 @@
         <f t="shared" si="13"/>
         <v>181.57239706970927</v>
       </c>
-    </row>
-    <row r="23" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AQ22">
+        <v>18914981</v>
+      </c>
+      <c r="AR22" s="4">
+        <f t="shared" si="14"/>
+        <v>1.8803777281087408</v>
+      </c>
+      <c r="AS22" s="6"/>
+    </row>
+    <row r="23" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>19</v>
       </c>
@@ -29433,8 +29712,16 @@
         <f t="shared" si="13"/>
         <v>282.84032714069679</v>
       </c>
-    </row>
-    <row r="24" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AQ23">
+        <v>13045096</v>
+      </c>
+      <c r="AR23" s="4">
+        <f t="shared" si="14"/>
+        <v>5.9357221288367672</v>
+      </c>
+      <c r="AS23" s="6"/>
+    </row>
+    <row r="24" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>20</v>
       </c>
@@ -29519,8 +29806,16 @@
         <f t="shared" si="13"/>
         <v>272.97635211267607</v>
       </c>
-    </row>
-    <row r="25" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AQ24">
+        <v>28218359</v>
+      </c>
+      <c r="AR24" s="4">
+        <f t="shared" si="14"/>
+        <v>3.4341686913827978</v>
+      </c>
+      <c r="AS24" s="6"/>
+    </row>
+    <row r="25" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>21</v>
       </c>
@@ -29605,8 +29900,16 @@
         <f t="shared" si="13"/>
         <v>291.45039442234565</v>
       </c>
-    </row>
-    <row r="26" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AQ25">
+        <v>46782944</v>
+      </c>
+      <c r="AR25" s="4">
+        <f t="shared" si="14"/>
+        <v>2.1346743804750723</v>
+      </c>
+      <c r="AS25" s="6"/>
+    </row>
+    <row r="26" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>22</v>
       </c>
@@ -29691,9 +29994,25 @@
         <f t="shared" si="13"/>
         <v>303.55061718369336</v>
       </c>
+      <c r="AQ26">
+        <v>91294378</v>
+      </c>
+      <c r="AR26" s="4">
+        <f t="shared" si="14"/>
+        <v>1.6377447908128582</v>
+      </c>
+      <c r="AS26" s="6"/>
+    </row>
+    <row r="27" spans="1:45" x14ac:dyDescent="0.2">
+      <c r="AR27" s="4">
+        <f>AVERAGE(AR5:AR26)</f>
+        <v>2.842343777478324</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="7">
+    <mergeCell ref="AN2:AO2"/>
+    <mergeCell ref="AQ2:AR2"/>
     <mergeCell ref="E2:H2"/>
     <mergeCell ref="K2:O2"/>
     <mergeCell ref="S2:W2"/>
@@ -30051,26 +30370,26 @@
       </c>
     </row>
     <row r="29" spans="3:22" x14ac:dyDescent="0.2">
-      <c r="I29" s="47" t="s">
+      <c r="I29" s="51" t="s">
         <v>21</v>
       </c>
-      <c r="J29" s="47"/>
-      <c r="K29" s="47"/>
-      <c r="L29" s="47"/>
+      <c r="J29" s="51"/>
+      <c r="K29" s="51"/>
+      <c r="L29" s="51"/>
       <c r="M29" s="21"/>
-      <c r="N29" s="47" t="s">
+      <c r="N29" s="51" t="s">
         <v>25</v>
       </c>
-      <c r="O29" s="47"/>
-      <c r="P29" s="47"/>
-      <c r="Q29" s="47"/>
+      <c r="O29" s="51"/>
+      <c r="P29" s="51"/>
+      <c r="Q29" s="51"/>
       <c r="R29" s="21"/>
-      <c r="S29" s="47" t="s">
+      <c r="S29" s="51" t="s">
         <v>26</v>
       </c>
-      <c r="T29" s="47"/>
-      <c r="U29" s="47"/>
-      <c r="V29" s="47"/>
+      <c r="T29" s="51"/>
+      <c r="U29" s="51"/>
+      <c r="V29" s="51"/>
     </row>
     <row r="30" spans="3:22" x14ac:dyDescent="0.2">
       <c r="I30" s="21" t="s">
@@ -30432,7 +30751,7 @@
       <c r="E9">
         <v>1</v>
       </c>
-      <c r="F9" s="56">
+      <c r="F9" s="46">
         <v>55.567</v>
       </c>
       <c r="G9" s="4">
@@ -30452,7 +30771,7 @@
       <c r="E10">
         <v>2</v>
       </c>
-      <c r="F10" s="56">
+      <c r="F10" s="46">
         <v>28.588000000000001</v>
       </c>
       <c r="G10" s="4">
@@ -30472,7 +30791,7 @@
       <c r="E11">
         <v>3</v>
       </c>
-      <c r="F11" s="56">
+      <c r="F11" s="46">
         <v>49.042000000000002</v>
       </c>
       <c r="G11" s="4">
@@ -30492,7 +30811,7 @@
       <c r="E12">
         <v>4</v>
       </c>
-      <c r="F12" s="56">
+      <c r="F12" s="46">
         <v>24.074999999999999</v>
       </c>
       <c r="G12" s="4">
@@ -30512,7 +30831,7 @@
       <c r="E13">
         <v>5</v>
       </c>
-      <c r="F13" s="56">
+      <c r="F13" s="46">
         <v>57.923000000000002</v>
       </c>
       <c r="G13" s="4">
@@ -30532,7 +30851,7 @@
       <c r="E14">
         <v>6</v>
       </c>
-      <c r="F14" s="56">
+      <c r="F14" s="46">
         <v>13.792</v>
       </c>
       <c r="G14" s="4">
@@ -30552,7 +30871,7 @@
       <c r="E15">
         <v>7</v>
       </c>
-      <c r="F15" s="56">
+      <c r="F15" s="46">
         <v>23.728000000000002</v>
       </c>
       <c r="G15" s="4">
@@ -30572,7 +30891,7 @@
       <c r="E16">
         <v>8</v>
       </c>
-      <c r="F16" s="56">
+      <c r="F16" s="46">
         <v>39.390999999999998</v>
       </c>
       <c r="G16" s="4">
@@ -30592,7 +30911,7 @@
       <c r="E17">
         <v>9</v>
       </c>
-      <c r="F17" s="56">
+      <c r="F17" s="46">
         <v>59.155000000000001</v>
       </c>
       <c r="G17" s="4">
@@ -30612,7 +30931,7 @@
       <c r="E18">
         <v>10</v>
       </c>
-      <c r="F18" s="56">
+      <c r="F18" s="46">
         <v>52.597000000000001</v>
       </c>
       <c r="G18" s="4">
@@ -30632,7 +30951,7 @@
       <c r="E19">
         <v>11</v>
       </c>
-      <c r="F19" s="56">
+      <c r="F19" s="46">
         <v>50.420999999999999</v>
       </c>
       <c r="G19" s="4">
@@ -30652,7 +30971,7 @@
       <c r="E20">
         <v>12</v>
       </c>
-      <c r="F20" s="56">
+      <c r="F20" s="46">
         <v>88.590999999999994</v>
       </c>
       <c r="G20" s="4">
@@ -30672,7 +30991,7 @@
       <c r="E21">
         <v>13</v>
       </c>
-      <c r="F21" s="56">
+      <c r="F21" s="46">
         <v>102.4</v>
       </c>
       <c r="G21" s="4">
@@ -30692,7 +31011,7 @@
       <c r="E22">
         <v>14</v>
       </c>
-      <c r="F22" s="56">
+      <c r="F22" s="46">
         <v>115.67</v>
       </c>
       <c r="G22" s="4">
@@ -30712,7 +31031,7 @@
       <c r="E23">
         <v>15</v>
       </c>
-      <c r="F23" s="56">
+      <c r="F23" s="46">
         <v>116.88</v>
       </c>
       <c r="G23" s="4">
@@ -30732,7 +31051,7 @@
       <c r="E24">
         <v>16</v>
       </c>
-      <c r="F24" s="57" t="s">
+      <c r="F24" s="47" t="s">
         <v>44</v>
       </c>
       <c r="G24" s="4">
@@ -30752,7 +31071,7 @@
       <c r="E25">
         <v>17</v>
       </c>
-      <c r="F25" s="57" t="s">
+      <c r="F25" s="47" t="s">
         <v>44</v>
       </c>
       <c r="G25" s="4">
@@ -30772,7 +31091,7 @@
       <c r="E26">
         <v>18</v>
       </c>
-      <c r="F26" s="57" t="s">
+      <c r="F26" s="47" t="s">
         <v>44</v>
       </c>
       <c r="G26" s="4">
@@ -30792,7 +31111,7 @@
       <c r="E27">
         <v>19</v>
       </c>
-      <c r="F27" s="57" t="s">
+      <c r="F27" s="47" t="s">
         <v>44</v>
       </c>
       <c r="G27" s="4">
@@ -30812,7 +31131,7 @@
       <c r="E28">
         <v>20</v>
       </c>
-      <c r="F28" s="57" t="s">
+      <c r="F28" s="47" t="s">
         <v>44</v>
       </c>
       <c r="G28" s="4">
@@ -30832,7 +31151,7 @@
       <c r="E29">
         <v>21</v>
       </c>
-      <c r="F29" s="57" t="s">
+      <c r="F29" s="47" t="s">
         <v>44</v>
       </c>
       <c r="G29" s="4">
@@ -30852,19 +31171,19 @@
       <c r="E30" s="33">
         <v>22</v>
       </c>
-      <c r="F30" s="58" t="s">
+      <c r="F30" s="48" t="s">
         <v>44</v>
       </c>
-      <c r="G30" s="59">
+      <c r="G30" s="49">
         <v>55.188527594611443</v>
       </c>
-      <c r="H30" s="59">
+      <c r="H30" s="49">
         <v>57.794670840440524</v>
       </c>
-      <c r="I30" s="59">
+      <c r="I30" s="49">
         <v>213.19553193450713</v>
       </c>
-      <c r="J30" s="59">
+      <c r="J30" s="49">
         <v>303.55061718369336</v>
       </c>
     </row>

</xml_diff>